<commit_message>
Refresh concert data with validated openers and headliner corrections
</commit_message>
<xml_diff>
--- a/Concert History.xlsx
+++ b/Concert History.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="426">
   <si>
     <t>Date</t>
   </si>
@@ -111,7 +111,7 @@
     <t>Snocore 99 Tour</t>
   </si>
   <si>
-    <t>Mr Bungle, Incubus</t>
+    <t>Mr. Bungle, Incubus</t>
   </si>
   <si>
     <t>Co-headline tour with Mr. Bungle</t>
@@ -546,7 +546,7 @@
     <t>The Getaway World Tour</t>
   </si>
   <si>
-    <t>Babymetal</t>
+    <t>BABYMETAL</t>
   </si>
   <si>
     <t>Metallica</t>
@@ -558,7 +558,7 @@
     <t>WorldWired Tour</t>
   </si>
   <si>
-    <t>Avenged Sevenfold, Volbeat</t>
+    <t>Volbeat, Local H, Mix Master Mike</t>
   </si>
   <si>
     <t>Fairfax</t>
@@ -666,7 +666,7 @@
     <t>Rock on the Range 2018</t>
   </si>
   <si>
-    <t>Alice in Chains, A Perfect Circle, Breaking Benjamin, Machine Gun Kelly, Greta Van Fleet, 10 Years, The Bronx, Underoath, Quicksand, Hawthorne Heights, Turnstile, Senses Fail, The Fever 333, I See Stars, Body Count, Atreyu, Power Trip, Dance Gavin Dance, Mutoid Man, Spirit Animal</t>
+    <t>Alice in Chains, A Perfect Circle, Breaking Benjamin, Machine Gun Kelly, Greta Van Fleet, 10 Years, The Bronx, Underoath, Quicksand, Hawthorne Heights, Turnstile, Senses Fail, Fever 333, I See Stars, Body Count, Atreyu, Power Trip, Dance Gavin Dance, Mutoid Man, Spirit Animal</t>
   </si>
   <si>
     <t>Glamping! First Festival!</t>
@@ -807,7 +807,7 @@
     <t>Ember Tour</t>
   </si>
   <si>
-    <t>Chevelle, Three Days Grace, Dorothy, Diamente</t>
+    <t>Chevelle, Three Days Grace, Dorothy, DIAMANTE</t>
   </si>
   <si>
     <t>Ghost</t>
@@ -840,7 +840,7 @@
     <t>Fear Inoculum Tour</t>
   </si>
   <si>
-    <t>Author and Punisher</t>
+    <t>Killing Joke</t>
   </si>
   <si>
     <t>Josh R., Bill B.</t>
@@ -855,6 +855,9 @@
     <t>T-Mobile Arena</t>
   </si>
   <si>
+    <t>Author &amp; Punisher</t>
+  </si>
+  <si>
     <t>Lily K.</t>
   </si>
   <si>
@@ -888,7 +891,7 @@
     <t>Welcome To Rockville Festival - Day 2</t>
   </si>
   <si>
-    <t>Metallica, Social Distortion, Pennywise, Ice Nine Kills, Ayron Jones, Austin Meade, Rob Zombie, Chevelle, Beartooth, Starset, Zero 9:36, Whit3 Collr, Wage War, Butcher Babies, Amigo the Devil, Bad Omens, Tallah, Eva Under Fire, Zero 9:36, Whit3 Collr, Divided Truth, ReBirth, Tragic, VENTRUSS, The Coursing, As You Were</t>
+    <t>Metallica, Social Distortion, Pennywise, Ice Nine Kills, Ayron Jones, Austin Meade, Rob Zombie, Chevelle, Beartooth, Starset, Wage War, Butcher Babies, Amigo the Devil, Bad Omens, Tallah, Eva Under Fire, Zero 9:36, Whit3 Collr, Divided Truth, ReBirth, Tragic, VENTRUSS, The Coursing, As You Were</t>
   </si>
   <si>
     <t>Welcome To Rockville Festival- Day 3</t>
@@ -945,7 +948,7 @@
     <t>Boy Harsher</t>
   </si>
   <si>
-    <t>Lunatic Luau</t>
+    <t>Lunatic Luau Festival</t>
   </si>
   <si>
     <t>Virginia Beach</t>
@@ -1053,7 +1056,7 @@
     <t>Blue Ridge Rock Fest 2023</t>
   </si>
   <si>
-    <t>Slipknot, Danzig, Motionless In White, Sleep Token, Knocked Loose, Lorna Shore, Polyphia, Testament, VV, Electric Callboy, Coal Chamber, Flyleaf, The Black Dahlia Murder, Job For Cowboy, After The Burial, Woe Is Me, Like Moths To Flames, The Acacia Strain, Of Mice &amp; Men, Chelsea Grin, Catch Your Breath, Black S. Cherry, Upon A Burning Body, Afterlife, Struggle Jennings, Angelmaker, Crown the Empire, Conquer Divide, TrustCompany, Savage Hands, Demun Jones, Archers, Starbenders, Oliver Anthony</t>
+    <t>Slipknot, Danzig, Motionless in White, Sleep Token, Knocked Loose, Lorna Shore, Polyphia, Testament, VV, Electric Callboy, Coal Chamber, Flyleaf, The Black Dahlia Murder, Job For Cowboy, After The Burial, Woe Is Me, Like Moths to Flames, The Acacia Strain, Of Mice &amp; Men, Chelsea Grin, Catch Your Breath, Black S. Cherry, Upon A Burning Body, Afterlife, Struggle Jennings, Angelmaker, Crown the Empire, Conquer Divide, TrustCompany, Savage Hands, Demun Jones, Archers, Starbenders, Oliver Anthony</t>
   </si>
   <si>
     <t>Blue Ride Disaster Shitshow: https://digitalbeatmag.com/a-2023-blue-ridge-rock-fest-review/</t>
@@ -1128,7 +1131,7 @@
     <t>Disturbed, Evanescence, Mudvayne, Theory of a Deadman, P.O.D., Drowning Pool, Nita Strauss, Judas Priest, Kerry King, The Ghost Inside, Nova Twins, Taipei Houston, Bob Vylan, Tim Montana, Cypress Hill, Electric Callboy, Enter Shikari, The Chats, Magnolia Park, TX2, Lø Spirit, Machine Head, August Burns Red, Frank Carter &amp; The Rattlesnakes, Fire from the Gods, Miss May I, Catch Your Breath, SiM, HotBox</t>
   </si>
   <si>
-    <t>The Original Misfits, Falling In Reverse, Seether, Anthrax, Dirty Honey, Nonpoint, Point North, Rise Against, Sum 41, Black Veil Brides, Movements, Terror, Scowl, Gel, Code Orange, Mr. Bungle, Drain, Militarie Gun, Rain City Drive, The Chisel, Gideon, Avatar, Atreyu, Soulfly, Kublai Khan TX, New Years Day, Fleshwater, I See Stars, Fuming Mouth</t>
+    <t>The Original Misfits, Falling in Reverse, Seether, Anthrax, Dirty Honey, Nonpoint, Point North, Rise Against, Sum 41, Black Veil Brides, Movements, Terror, Scowl, Gel, Code Orange, Mr. Bungle, Drain, Militarie Gun, Rain City Drive, The Chisel, Gideon, Avatar, Atreyu, Soulfly, Kublai Khan TX, New Years Day, Fleshwater, I See Stars, Fuming Mouth</t>
   </si>
   <si>
     <t>Pantera, Staind, Breaking Benjamin, Starset, Living Colour, Saint Asonia, Flat Black, Sleep Token, In This Moment, Flyleaf with Lacey Sturm, Kittie, Destroy Boys, Calva Louise, VUKOVI, Polyphia, The Amity Affliction, Currents, Spite, Bodysnatcher, Thrown, Dying Wish, Slaughter to Prevail, In Flames, Lacuna Coil, Harm's Way, Empire State Bastard, Imminence, Mike's Dead</t>
@@ -1140,7 +1143,7 @@
     <t>Unlimited Love Tour</t>
   </si>
   <si>
-    <t>IRONTOM</t>
+    <t>Ice Cube</t>
   </si>
   <si>
     <t>Loaded: The Greatest Hits 1994-2023 Tour</t>
@@ -1152,7 +1155,7 @@
     <t>Jubilee Tour</t>
   </si>
   <si>
-    <t>LIVE, Soul Asylum</t>
+    <t>Live, Soul Asylum</t>
   </si>
   <si>
     <t>Co-headline tour with Live.</t>
@@ -1179,13 +1182,13 @@
     <t>From Zero World Tour</t>
   </si>
   <si>
-    <t>Jean Dawson</t>
+    <t>grandson</t>
   </si>
   <si>
     <t>Dark Matter World Tour</t>
   </si>
   <si>
-    <t>Teen Jesus and the Jean Teaser</t>
+    <t>Teen Jesus and the Jean Teasers</t>
   </si>
   <si>
     <t>Bank of America Stadium</t>
@@ -1239,7 +1242,7 @@
     <t>I Can't Hear You Tour</t>
   </si>
   <si>
-    <t>Health, Daycare, Destroy Boys</t>
+    <t>Health, Ecca Vandal, Like Roses</t>
   </si>
   <si>
     <t>Co-headline tour with Health.</t>
@@ -1248,7 +1251,7 @@
     <t>Lucro Sucio: Los Ojos del Vacio Tour</t>
   </si>
   <si>
-    <t>Teri Gender Bender</t>
+    <t>Feliz y Dada, Kianî Medina</t>
   </si>
   <si>
     <t>Candlebox</t>
@@ -1842,7 +1845,7 @@
       <c r="J4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="7" t="s">
         <v>32</v>
       </c>
       <c r="L4" s="15" t="s">
@@ -2949,7 +2952,7 @@
       <c r="J35" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="K35" s="21" t="s">
+      <c r="K35" s="22" t="s">
         <v>177</v>
       </c>
       <c r="L35" s="9"/>
@@ -2985,7 +2988,7 @@
       <c r="J36" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="K36" s="21" t="s">
+      <c r="K36" s="22" t="s">
         <v>181</v>
       </c>
       <c r="L36" s="9"/>
@@ -4010,7 +4013,7 @@
         <v>274</v>
       </c>
       <c r="K65" s="28" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="L65" s="9"/>
     </row>
@@ -4034,7 +4037,7 @@
         <v>163</v>
       </c>
       <c r="G66" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H66" s="11" t="s">
         <v>85</v>
@@ -4046,7 +4049,7 @@
         <v>242</v>
       </c>
       <c r="K66" s="28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L66" s="9"/>
     </row>
@@ -4058,7 +4061,7 @@
         <v>62</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D67" s="11" t="s">
         <v>75</v>
@@ -4079,7 +4082,7 @@
         <v>27</v>
       </c>
       <c r="J67" s="21" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L67" s="9"/>
     </row>
@@ -4112,7 +4115,7 @@
         <v>27</v>
       </c>
       <c r="J68" s="21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L68" s="9"/>
     </row>
@@ -4124,16 +4127,16 @@
         <v>37</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E69" s="19" t="s">
         <v>116</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G69" s="13" t="s">
         <v>164</v>
@@ -4145,10 +4148,10 @@
         <v>27</v>
       </c>
       <c r="J69" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K69" s="28" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L69" s="7"/>
     </row>
@@ -4160,16 +4163,16 @@
         <v>12</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E70" s="19" t="s">
         <v>116</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G70" s="13" t="s">
         <v>164</v>
@@ -4181,10 +4184,10 @@
         <v>27</v>
       </c>
       <c r="J70" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K70" s="28" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L70" s="7"/>
     </row>
@@ -4196,16 +4199,16 @@
         <v>62</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D71" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E71" s="19" t="s">
         <v>116</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G71" s="13" t="s">
         <v>164</v>
@@ -4217,10 +4220,10 @@
         <v>27</v>
       </c>
       <c r="J71" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K71" s="28" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L71" s="7"/>
     </row>
@@ -4232,16 +4235,16 @@
         <v>21</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E72" s="19" t="s">
         <v>116</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G72" s="13" t="s">
         <v>164</v>
@@ -4253,10 +4256,10 @@
         <v>27</v>
       </c>
       <c r="J72" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K72" s="28" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L72" s="7"/>
     </row>
@@ -4268,7 +4271,7 @@
         <v>12</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>75</v>
@@ -4280,7 +4283,7 @@
         <v>103</v>
       </c>
       <c r="G73" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H73" s="11" t="s">
         <v>85</v>
@@ -4289,7 +4292,7 @@
         <v>27</v>
       </c>
       <c r="J73" s="21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L73" s="9"/>
     </row>
@@ -4304,13 +4307,13 @@
         <v>144</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E74" s="19" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G74" s="13" t="s">
         <v>233</v>
@@ -4325,7 +4328,7 @@
         <v>274</v>
       </c>
       <c r="K74" s="28" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L74" s="9"/>
     </row>
@@ -4337,7 +4340,7 @@
         <v>12</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D75" s="11" t="s">
         <v>162</v>
@@ -4358,10 +4361,10 @@
         <v>27</v>
       </c>
       <c r="J75" s="21" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K75" s="28" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L75" s="9"/>
     </row>
@@ -4376,13 +4379,13 @@
         <v>144</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E76" s="19" t="s">
         <v>213</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G76" s="13" t="s">
         <v>233</v>
@@ -4397,7 +4400,7 @@
         <v>274</v>
       </c>
       <c r="K76" s="28" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L76" s="9"/>
     </row>
@@ -4430,10 +4433,10 @@
         <v>27</v>
       </c>
       <c r="J77" s="21" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K77" s="28" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L77" s="9"/>
     </row>
@@ -4444,20 +4447,20 @@
       <c r="B78" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C78" s="11" t="s">
-        <v>310</v>
+      <c r="C78" s="13" t="s">
+        <v>311</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E78" s="19" t="s">
         <v>183</v>
       </c>
       <c r="F78" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H78" s="11" t="s">
         <v>18</v>
@@ -4466,10 +4469,10 @@
         <v>27</v>
       </c>
       <c r="J78" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K78" s="22" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L78" s="9"/>
     </row>
@@ -4502,10 +4505,10 @@
         <v>27</v>
       </c>
       <c r="J79" s="21" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K79" s="28" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L79" s="9"/>
     </row>
@@ -4517,7 +4520,7 @@
         <v>21</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D80" s="11" t="s">
         <v>75</v>
@@ -4529,7 +4532,7 @@
         <v>103</v>
       </c>
       <c r="G80" s="13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H80" s="11" t="s">
         <v>85</v>
@@ -4538,10 +4541,10 @@
         <v>27</v>
       </c>
       <c r="J80" s="21" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="K80" s="28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L80" s="9"/>
     </row>
@@ -4565,7 +4568,7 @@
         <v>103</v>
       </c>
       <c r="G81" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="H81" s="11" t="s">
         <v>18</v>
@@ -4574,7 +4577,7 @@
         <v>27</v>
       </c>
       <c r="J81" s="21" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L81" s="9"/>
     </row>
@@ -4586,16 +4589,16 @@
         <v>21</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E82" s="19" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G82" s="13" t="s">
         <v>233</v>
@@ -4607,10 +4610,10 @@
         <v>27</v>
       </c>
       <c r="J82" s="21" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K82" s="28" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L82" s="9"/>
     </row>
@@ -4622,7 +4625,7 @@
         <v>29</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D83" s="11" t="s">
         <v>75</v>
@@ -4643,13 +4646,13 @@
         <v>27</v>
       </c>
       <c r="J83" s="21" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K83" s="28" t="s">
         <v>261</v>
       </c>
       <c r="L83" s="23" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
@@ -4681,10 +4684,10 @@
         <v>27</v>
       </c>
       <c r="J84" s="21" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="K84" s="28" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="L84" s="9"/>
     </row>
@@ -4696,16 +4699,16 @@
         <v>21</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D85" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E85" s="19" t="s">
         <v>116</v>
       </c>
       <c r="F85" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G85" s="13" t="s">
         <v>164</v>
@@ -4717,10 +4720,10 @@
         <v>27</v>
       </c>
       <c r="J85" s="22" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K85" s="28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="L85" s="7"/>
     </row>
@@ -4735,13 +4738,13 @@
         <v>178</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E86" s="19" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F86" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G86" s="13" t="s">
         <v>233</v>
@@ -4753,10 +4756,10 @@
         <v>27</v>
       </c>
       <c r="J86" s="21" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K86" s="28" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="L86" s="9"/>
     </row>
@@ -4768,16 +4771,16 @@
         <v>37</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D87" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E87" s="19" t="s">
         <v>183</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G87" s="13" t="s">
         <v>164</v>
@@ -4789,13 +4792,13 @@
         <v>27</v>
       </c>
       <c r="J87" s="22" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K87" s="28" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="L87" s="7" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
@@ -4806,7 +4809,7 @@
         <v>62</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D88" s="11" t="s">
         <v>277</v>
@@ -4815,7 +4818,7 @@
         <v>278</v>
       </c>
       <c r="F88" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G88" s="13" t="s">
         <v>231</v>
@@ -4827,7 +4830,7 @@
         <v>27</v>
       </c>
       <c r="J88" s="21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L88" s="9"/>
     </row>
@@ -4839,7 +4842,7 @@
         <v>21</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D89" s="11" t="s">
         <v>75</v>
@@ -4860,10 +4863,10 @@
         <v>27</v>
       </c>
       <c r="J89" s="21" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K89" s="9" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="L89" s="9"/>
     </row>
@@ -4875,7 +4878,7 @@
         <v>37</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D90" s="11" t="s">
         <v>75</v>
@@ -4896,10 +4899,10 @@
         <v>27</v>
       </c>
       <c r="J90" s="21" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="K90" s="28" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="L90" s="9"/>
     </row>
@@ -4911,7 +4914,7 @@
         <v>12</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D91" s="11" t="s">
         <v>129</v>
@@ -4923,7 +4926,7 @@
         <v>130</v>
       </c>
       <c r="G91" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H91" s="11" t="s">
         <v>18</v>
@@ -4932,10 +4935,10 @@
         <v>27</v>
       </c>
       <c r="J91" s="21" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K91" s="28" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L91" s="9"/>
     </row>
@@ -4968,10 +4971,10 @@
         <v>27</v>
       </c>
       <c r="J92" s="21" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K92" s="28" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L92" s="9"/>
     </row>
@@ -5004,10 +5007,10 @@
         <v>27</v>
       </c>
       <c r="J93" s="21" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K93" s="28" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L93" s="9"/>
     </row>
@@ -5019,7 +5022,7 @@
         <v>12</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D94" s="11" t="s">
         <v>75</v>
@@ -5028,7 +5031,7 @@
         <v>76</v>
       </c>
       <c r="F94" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G94" s="13" t="s">
         <v>164</v>
@@ -5040,10 +5043,10 @@
         <v>27</v>
       </c>
       <c r="J94" s="21" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K94" s="28" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="L94" s="9"/>
     </row>
@@ -5055,7 +5058,7 @@
         <v>21</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D95" s="11" t="s">
         <v>75</v>
@@ -5076,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="J95" s="21" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="L95" s="21"/>
     </row>
@@ -5088,7 +5091,7 @@
         <v>37</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D96" s="11" t="s">
         <v>212</v>
@@ -5097,7 +5100,7 @@
         <v>213</v>
       </c>
       <c r="F96" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G96" s="13" t="s">
         <v>164</v>
@@ -5109,10 +5112,10 @@
         <v>27</v>
       </c>
       <c r="J96" s="29" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K96" s="28" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="L96" s="30"/>
     </row>
@@ -5124,7 +5127,7 @@
         <v>12</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D97" s="11" t="s">
         <v>212</v>
@@ -5133,7 +5136,7 @@
         <v>213</v>
       </c>
       <c r="F97" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G97" s="13" t="s">
         <v>164</v>
@@ -5145,10 +5148,10 @@
         <v>27</v>
       </c>
       <c r="J97" s="29" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K97" s="28" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="L97" s="30"/>
     </row>
@@ -5160,7 +5163,7 @@
         <v>62</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D98" s="11" t="s">
         <v>212</v>
@@ -5169,7 +5172,7 @@
         <v>213</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G98" s="13" t="s">
         <v>164</v>
@@ -5181,10 +5184,10 @@
         <v>27</v>
       </c>
       <c r="J98" s="29" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K98" s="28" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="L98" s="30"/>
     </row>
@@ -5196,7 +5199,7 @@
         <v>21</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D99" s="11" t="s">
         <v>212</v>
@@ -5205,7 +5208,7 @@
         <v>213</v>
       </c>
       <c r="F99" s="11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G99" s="13" t="s">
         <v>164</v>
@@ -5217,10 +5220,10 @@
         <v>27</v>
       </c>
       <c r="J99" s="29" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K99" s="28" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L99" s="30"/>
     </row>
@@ -5253,10 +5256,10 @@
         <v>27</v>
       </c>
       <c r="J100" s="21" t="s">
-        <v>374</v>
-      </c>
-      <c r="K100" s="21" t="s">
         <v>375</v>
+      </c>
+      <c r="K100" s="22" t="s">
+        <v>376</v>
       </c>
       <c r="L100" s="9"/>
     </row>
@@ -5268,7 +5271,7 @@
         <v>29</v>
       </c>
       <c r="C101" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D101" s="11" t="s">
         <v>75</v>
@@ -5289,10 +5292,10 @@
         <v>27</v>
       </c>
       <c r="J101" s="21" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K101" s="21" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L101" s="9"/>
     </row>
@@ -5325,13 +5328,13 @@
         <v>27</v>
       </c>
       <c r="J102" s="21" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K102" s="22" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L102" s="23" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
@@ -5342,7 +5345,7 @@
         <v>89</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D103" s="11" t="s">
         <v>75</v>
@@ -5363,10 +5366,10 @@
         <v>27</v>
       </c>
       <c r="J103" s="21" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K103" s="21" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="L103" s="9"/>
     </row>
@@ -5378,7 +5381,7 @@
         <v>54</v>
       </c>
       <c r="C104" s="9" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D104" s="9" t="s">
         <v>140</v>
@@ -5399,7 +5402,7 @@
         <v>27</v>
       </c>
       <c r="J104" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K104" s="9" t="s">
         <v>71</v>
@@ -5414,7 +5417,7 @@
         <v>29</v>
       </c>
       <c r="C105" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D105" s="11" t="s">
         <v>75</v>
@@ -5423,7 +5426,7 @@
         <v>76</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G105" s="13" t="s">
         <v>276</v>
@@ -5435,10 +5438,10 @@
         <v>27</v>
       </c>
       <c r="J105" s="21" t="s">
-        <v>387</v>
-      </c>
-      <c r="K105" s="21" t="s">
         <v>388</v>
+      </c>
+      <c r="K105" s="22" t="s">
+        <v>389</v>
       </c>
       <c r="L105" s="9"/>
     </row>
@@ -5459,7 +5462,7 @@
         <v>76</v>
       </c>
       <c r="F106" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G106" s="13" t="s">
         <v>164</v>
@@ -5471,10 +5474,10 @@
         <v>27</v>
       </c>
       <c r="J106" s="21" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K106" s="22" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="L106" s="9"/>
     </row>
@@ -5495,7 +5498,7 @@
         <v>76</v>
       </c>
       <c r="F107" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G107" s="13" t="s">
         <v>276</v>
@@ -5507,10 +5510,10 @@
         <v>27</v>
       </c>
       <c r="J107" s="21" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K107" s="21" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="L107" s="9"/>
     </row>
@@ -5531,10 +5534,10 @@
         <v>76</v>
       </c>
       <c r="F108" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G108" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H108" s="11" t="s">
         <v>18</v>
@@ -5543,7 +5546,7 @@
         <v>27</v>
       </c>
       <c r="J108" s="21" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K108" s="9"/>
       <c r="L108" s="9"/>
@@ -5556,7 +5559,7 @@
         <v>29</v>
       </c>
       <c r="C109" s="11" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D109" s="11" t="s">
         <v>129</v>
@@ -5577,7 +5580,7 @@
         <v>27</v>
       </c>
       <c r="J109" s="21" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K109" s="9"/>
       <c r="L109" s="9"/>
@@ -5590,7 +5593,7 @@
         <v>37</v>
       </c>
       <c r="C110" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D110" s="11" t="s">
         <v>75</v>
@@ -5599,10 +5602,10 @@
         <v>76</v>
       </c>
       <c r="F110" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G110" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H110" s="11" t="s">
         <v>18</v>
@@ -5611,10 +5614,10 @@
         <v>27</v>
       </c>
       <c r="J110" s="21" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K110" s="21" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L110" s="9"/>
     </row>
@@ -5629,13 +5632,13 @@
         <v>30</v>
       </c>
       <c r="D111" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E111" s="19" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F111" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G111" s="13" t="s">
         <v>233</v>
@@ -5647,10 +5650,10 @@
         <v>27</v>
       </c>
       <c r="J111" s="21" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K111" s="21" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L111" s="9"/>
     </row>
@@ -5671,7 +5674,7 @@
         <v>76</v>
       </c>
       <c r="F112" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G112" s="13" t="s">
         <v>276</v>
@@ -5683,10 +5686,10 @@
         <v>27</v>
       </c>
       <c r="J112" s="21" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K112" s="21" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="L112" s="9"/>
     </row>
@@ -5698,7 +5701,7 @@
         <v>37</v>
       </c>
       <c r="C113" s="13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D113" s="11" t="s">
         <v>75</v>
@@ -5707,7 +5710,7 @@
         <v>76</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G113" s="13" t="s">
         <v>69</v>
@@ -5719,10 +5722,10 @@
         <v>27</v>
       </c>
       <c r="J113" s="21" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K113" s="22" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L113" s="9"/>
     </row>
@@ -5734,7 +5737,7 @@
         <v>62</v>
       </c>
       <c r="C114" s="11" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D114" s="11" t="s">
         <v>75</v>
@@ -5755,13 +5758,13 @@
         <v>27</v>
       </c>
       <c r="J114" s="21" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K114" s="22" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="L114" s="23" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
@@ -5793,10 +5796,10 @@
         <v>27</v>
       </c>
       <c r="J115" s="21" t="s">
-        <v>410</v>
-      </c>
-      <c r="K115" s="21" t="s">
         <v>411</v>
+      </c>
+      <c r="K115" s="22" t="s">
+        <v>412</v>
       </c>
       <c r="L115" s="9"/>
     </row>
@@ -5829,10 +5832,10 @@
         <v>27</v>
       </c>
       <c r="J116" s="21" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K116" s="9" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="L116" s="9"/>
     </row>
@@ -5844,16 +5847,16 @@
         <v>62</v>
       </c>
       <c r="C117" s="11" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D117" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E117" s="19" t="s">
         <v>183</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G117" s="13" t="s">
         <v>164</v>
@@ -5865,10 +5868,10 @@
         <v>27</v>
       </c>
       <c r="J117" s="21" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K117" s="9" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="L117" s="9"/>
     </row>
@@ -5880,7 +5883,7 @@
         <v>54</v>
       </c>
       <c r="C118" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D118" s="11" t="s">
         <v>75</v>
@@ -5889,7 +5892,7 @@
         <v>76</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G118" s="13" t="s">
         <v>233</v>
@@ -5901,10 +5904,10 @@
         <v>27</v>
       </c>
       <c r="J118" s="21" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K118" s="21" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="L118" s="9"/>
     </row>
@@ -5937,7 +5940,7 @@
         <v>27</v>
       </c>
       <c r="J119" s="7" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K119" s="9"/>
       <c r="L119" s="9"/>
@@ -5971,10 +5974,10 @@
         <v>27</v>
       </c>
       <c r="J120" s="21" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K120" s="7" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="L120" s="9"/>
     </row>
@@ -5986,7 +5989,7 @@
         <v>12</v>
       </c>
       <c r="C121" s="9" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D121" s="9" t="s">
         <v>162</v>
@@ -5995,7 +5998,7 @@
         <v>76</v>
       </c>
       <c r="F121" s="9" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G121" s="7" t="s">
         <v>164</v>
@@ -6007,7 +6010,7 @@
         <v>27</v>
       </c>
       <c r="J121" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K121" s="9"/>
       <c r="L121" s="9"/>

</xml_diff>

<commit_message>
Move festival_images to images/festivals/ for org consistency
</commit_message>
<xml_diff>
--- a/Concert History.xlsx
+++ b/Concert History.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="427">
   <si>
     <t>Date</t>
   </si>
@@ -75,7 +75,7 @@
     <t>College and University Independant Tour</t>
   </si>
   <si>
-    <t>Greg Humphrys</t>
+    <t>Hobex</t>
   </si>
   <si>
     <t>Sunday</t>
@@ -591,7 +591,7 @@
     <t>2017 Summer Tour</t>
   </si>
   <si>
-    <t>Clutch, The Fungi Band</t>
+    <t>Clutch</t>
   </si>
   <si>
     <t>Winston Salem</t>
@@ -768,7 +768,7 @@
     <t>Motionless in White, Badflower, The Damned Things, Wage War, Crobot, Sylar, Shvpes, Dirty Honey, Alien Weaponry, Hyde, Tetrarch, Dead Girls Academy</t>
   </si>
   <si>
-    <t>Note: Tool, Judas Priest, The Cult, Bush, Black Label Society, Circa Survive, Yelawolf, Grandson, Memphis May Fire, and Starset were all cancelled or cut short due to the storm evacuation.</t>
+    <t>Note: Tool, Judas Priest, The Cult, Bush, Black Label Society, Circa Survive, Yelawolf, grandson, Memphis May Fire, and Starset were all cancelled or cut short due to the storm evacuation.</t>
   </si>
   <si>
     <t>Epicenter Festival - Day 3</t>
@@ -885,7 +885,7 @@
     <t>Welcome to Rockville 2021</t>
   </si>
   <si>
-    <t>Slipknot, Cypress Hill, Grandson, Dead Sara, Spiritbox, Dana Dentata, A Day to Remember, Gojira, Dorothy, Teenage Wrist, Siiickbrain, Brass Against, NASCAR Aloe, Jeris Johnson, Blame My Youth, Contracult Collective, Them Evils, Revision, Revised, The Alpha Complex, A War Within, Scarlett O'hara, Dead Reckoning, Shadow the Earth, As You Were</t>
+    <t>Slipknot, Cypress Hill, grandson, Dead Sara, Spiritbox, Dana Dentata, A Day to Remember, Gojira, Dorothy, Teenage Wrist, Siiickbrain, Brass Against, NASCAR Aloe, Jeris Johnson, Blame My Youth, Contracult Collective, Them Evils, Revision, Revised, The Alpha Complex, A War Within, Scarlett O'hara, Dead Reckoning, Shadow the Earth, As You Were</t>
   </si>
   <si>
     <t>Welcome To Rockville Festival - Day 2</t>
@@ -1026,7 +1026,7 @@
     <t>Welcome to Rockville 2023</t>
   </si>
   <si>
-    <t>Tool, Deftones, Incubus, The Mars Volta, Coheed &amp; Cambria, Pennywise, Ghostemane, Grandson, Sueco, Filter, Deafheaven, Anti-Flag, Senses Fail, New Years Day, Nothing,Nowhere, Angel Dust, Nova Twins, Point North, Bob Vylan, Capital Theatre, Uncured, Reddstar</t>
+    <t>Tool, Deftones, Incubus, The Mars Volta, Coheed &amp; Cambria, Pennywise, Ghostemane, grandson, Sueco, Filter, Deafheaven, Anti-Flag, Senses Fail, New Years Day, Nothing,Nowhere, Angel Dust, Nova Twins, Point North, Bob Vylan, Capital Theatre, Uncured, Reddstar</t>
   </si>
   <si>
     <t>East Rutherford</t>
@@ -1281,7 +1281,10 @@
     <t>Normal Isn't Tour</t>
   </si>
   <si>
-    <t>Dave Hill, Puddles Pity Party (guest appearance)</t>
+    <t>Dave Hill</t>
+  </si>
+  <si>
+    <t>Puddles Pity Party (guest appearance)</t>
   </si>
   <si>
     <t>AVTT/PTTN</t>
@@ -3096,7 +3099,7 @@
       <c r="J39" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="K39" s="21" t="s">
+      <c r="K39" s="22" t="s">
         <v>192</v>
       </c>
       <c r="L39" s="9"/>
@@ -5979,7 +5982,9 @@
       <c r="K120" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="L120" s="9"/>
+      <c r="L120" s="7" t="s">
+        <v>423</v>
+      </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="10">
@@ -5989,7 +5994,7 @@
         <v>12</v>
       </c>
       <c r="C121" s="9" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D121" s="9" t="s">
         <v>162</v>
@@ -5998,7 +6003,7 @@
         <v>76</v>
       </c>
       <c r="F121" s="9" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G121" s="7" t="s">
         <v>164</v>
@@ -6010,7 +6015,7 @@
         <v>27</v>
       </c>
       <c r="J121" s="7" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K121" s="9"/>
       <c r="L121" s="9"/>

</xml_diff>

<commit_message>
Add new shows, refresh setlists, brand polish
</commit_message>
<xml_diff>
--- a/Concert History.xlsx
+++ b/Concert History.xlsx
@@ -3090,8 +3090,8 @@
       <c r="G39" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="H39" s="11" t="s">
-        <v>18</v>
+      <c r="H39" s="13" t="s">
+        <v>85</v>
       </c>
       <c r="I39" s="20" t="s">
         <v>27</v>
@@ -3590,8 +3590,8 @@
       <c r="G53" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="H53" s="11" t="s">
-        <v>18</v>
+      <c r="H53" s="13" t="s">
+        <v>85</v>
       </c>
       <c r="I53" s="20" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Add <artist> <date> concert and poster
</commit_message>
<xml_diff>
--- a/Concert History.xlsx
+++ b/Concert History.xlsx
@@ -1236,7 +1236,7 @@
     <t>Rob Schneider</t>
   </si>
   <si>
-    <t>Pierce the Veil</t>
+    <t>Health</t>
   </si>
   <si>
     <t>Co-Headline tour with Pierce the Veil</t>
@@ -5770,7 +5770,7 @@
       <c r="B114" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="C114" s="11" t="s">
+      <c r="C114" s="13" t="s">
         <v>407</v>
       </c>
       <c r="D114" s="11" t="s">

</xml_diff>